<commit_message>
Merge product-like categories into Products
</commit_message>
<xml_diff>
--- a/source/Inventory_Master_V7.xlsx
+++ b/source/Inventory_Master_V7.xlsx
@@ -2048,12 +2048,12 @@
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B19" s="16" t="inlineStr">
         <is>
-          <t>CHM-0018</t>
+          <t>PRD-0001</t>
         </is>
       </c>
       <c r="C19" s="15" t="inlineStr">
@@ -2675,12 +2675,12 @@
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>CHM-0027</t>
+          <t>PRD-0002</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
@@ -6611,12 +6611,12 @@
     <row r="84" ht="16" customHeight="1">
       <c r="A84" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t>CHM-0083</t>
+          <t>PRD-0003</t>
         </is>
       </c>
       <c r="C84" s="9" t="inlineStr">
@@ -8240,12 +8240,12 @@
     <row r="107" ht="16" customHeight="1">
       <c r="A107" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B107" s="16" t="inlineStr">
         <is>
-          <t>CHM-0106</t>
+          <t>PRD-0004</t>
         </is>
       </c>
       <c r="C107" s="15" t="inlineStr">
@@ -11253,12 +11253,12 @@
     <row r="150" ht="16" customHeight="1">
       <c r="A150" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B150" s="10" t="inlineStr">
         <is>
-          <t>CHM-0149</t>
+          <t>PRD-0005</t>
         </is>
       </c>
       <c r="C150" s="9" t="inlineStr">
@@ -11312,12 +11312,12 @@
     <row r="151" ht="16" customHeight="1">
       <c r="A151" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B151" s="16" t="inlineStr">
         <is>
-          <t>CHM-0150</t>
+          <t>PRD-0006</t>
         </is>
       </c>
       <c r="C151" s="15" t="inlineStr">
@@ -11900,12 +11900,12 @@
     <row r="159" ht="16" customHeight="1">
       <c r="A159" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B159" s="16" t="inlineStr">
         <is>
-          <t>CHM-0158</t>
+          <t>PRD-0007</t>
         </is>
       </c>
       <c r="C159" s="15" t="inlineStr">
@@ -15843,12 +15843,12 @@
     <row r="212" ht="16" customHeight="1">
       <c r="A212" s="9" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B212" s="10" t="inlineStr">
         <is>
-          <t>CHM-0211</t>
+          <t>PRD-0008</t>
         </is>
       </c>
       <c r="C212" s="9" t="inlineStr">
@@ -16364,12 +16364,12 @@
     <row r="219" ht="16" customHeight="1">
       <c r="A219" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B219" s="16" t="inlineStr">
         <is>
-          <t>CHM-0218</t>
+          <t>PRD-0009</t>
         </is>
       </c>
       <c r="C219" s="15" t="inlineStr">
@@ -19979,12 +19979,12 @@
     <row r="268" ht="16" customHeight="1">
       <c r="A268" s="9" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B268" s="10" t="inlineStr">
         <is>
-          <t>CHM-0267</t>
+          <t>PRD-0010</t>
         </is>
       </c>
       <c r="C268" s="9" t="inlineStr">
@@ -20050,12 +20050,12 @@
     <row r="269" ht="16" customHeight="1">
       <c r="A269" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B269" s="16" t="inlineStr">
         <is>
-          <t>CHM-0268</t>
+          <t>PRD-0011</t>
         </is>
       </c>
       <c r="C269" s="15" t="inlineStr">
@@ -20121,12 +20121,12 @@
     <row r="270" ht="16" customHeight="1">
       <c r="A270" s="9" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B270" s="10" t="inlineStr">
         <is>
-          <t>CHM-0269</t>
+          <t>PRD-0012</t>
         </is>
       </c>
       <c r="C270" s="9" t="inlineStr">
@@ -20192,12 +20192,12 @@
     <row r="271" ht="16" customHeight="1">
       <c r="A271" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B271" s="16" t="inlineStr">
         <is>
-          <t>CHM-0270</t>
+          <t>PRD-0013</t>
         </is>
       </c>
       <c r="C271" s="15" t="inlineStr">
@@ -20263,12 +20263,12 @@
     <row r="272" ht="16" customHeight="1">
       <c r="A272" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B272" s="10" t="inlineStr">
         <is>
-          <t>CHM-0271</t>
+          <t>PRD-0014</t>
         </is>
       </c>
       <c r="C272" s="9" t="inlineStr">
@@ -20334,12 +20334,12 @@
     <row r="273" ht="16" customHeight="1">
       <c r="A273" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B273" s="16" t="inlineStr">
         <is>
-          <t>CHM-0272</t>
+          <t>PRD-0015</t>
         </is>
       </c>
       <c r="C273" s="15" t="inlineStr">
@@ -20405,12 +20405,12 @@
     <row r="274" ht="16" customHeight="1">
       <c r="A274" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B274" s="10" t="inlineStr">
         <is>
-          <t>CHM-0273</t>
+          <t>PRD-0016</t>
         </is>
       </c>
       <c r="C274" s="9" t="inlineStr">
@@ -20476,12 +20476,12 @@
     <row r="275" ht="16" customHeight="1">
       <c r="A275" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B275" s="16" t="inlineStr">
         <is>
-          <t>CHM-0274</t>
+          <t>PRD-0017</t>
         </is>
       </c>
       <c r="C275" s="15" t="inlineStr">
@@ -20547,12 +20547,12 @@
     <row r="276" ht="16" customHeight="1">
       <c r="A276" s="9" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B276" s="10" t="inlineStr">
         <is>
-          <t>CHM-0275</t>
+          <t>PRD-0018</t>
         </is>
       </c>
       <c r="C276" s="9" t="inlineStr">
@@ -20618,12 +20618,12 @@
     <row r="277" ht="16" customHeight="1">
       <c r="A277" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B277" s="16" t="inlineStr">
         <is>
-          <t>CHM-0276</t>
+          <t>PRD-0019</t>
         </is>
       </c>
       <c r="C277" s="15" t="inlineStr">
@@ -20689,12 +20689,12 @@
     <row r="278" ht="16" customHeight="1">
       <c r="A278" s="9" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B278" s="10" t="inlineStr">
         <is>
-          <t>CHM-0277</t>
+          <t>PRD-0020</t>
         </is>
       </c>
       <c r="C278" s="9" t="inlineStr">
@@ -20760,12 +20760,12 @@
     <row r="279" ht="16" customHeight="1">
       <c r="A279" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B279" s="16" t="inlineStr">
         <is>
-          <t>CHM-0278</t>
+          <t>PRD-0021</t>
         </is>
       </c>
       <c r="C279" s="15" t="inlineStr">
@@ -20831,12 +20831,12 @@
     <row r="280" ht="16" customHeight="1">
       <c r="A280" s="9" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B280" s="10" t="inlineStr">
         <is>
-          <t>CHM-0279</t>
+          <t>PRD-0022</t>
         </is>
       </c>
       <c r="C280" s="9" t="inlineStr">
@@ -20902,12 +20902,12 @@
     <row r="281" ht="16" customHeight="1">
       <c r="A281" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B281" s="16" t="inlineStr">
         <is>
-          <t>CHM-0280</t>
+          <t>PRD-0023</t>
         </is>
       </c>
       <c r="C281" s="15" t="inlineStr">
@@ -21573,12 +21573,12 @@
     <row r="290" ht="16" customHeight="1">
       <c r="A290" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B290" s="10" t="inlineStr">
         <is>
-          <t>CHM-0289</t>
+          <t>PRD-0024</t>
         </is>
       </c>
       <c r="C290" s="9" t="inlineStr">
@@ -21644,12 +21644,12 @@
     <row r="291" ht="16" customHeight="1">
       <c r="A291" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B291" s="16" t="inlineStr">
         <is>
-          <t>CHM-0290</t>
+          <t>PRD-0025</t>
         </is>
       </c>
       <c r="C291" s="15" t="inlineStr">
@@ -21715,12 +21715,12 @@
     <row r="292" ht="16" customHeight="1">
       <c r="A292" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B292" s="10" t="inlineStr">
         <is>
-          <t>CHM-0291</t>
+          <t>PRD-0026</t>
         </is>
       </c>
       <c r="C292" s="9" t="inlineStr">
@@ -21786,12 +21786,12 @@
     <row r="293" ht="16" customHeight="1">
       <c r="A293" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B293" s="16" t="inlineStr">
         <is>
-          <t>CHM-0292</t>
+          <t>PRD-0027</t>
         </is>
       </c>
       <c r="C293" s="15" t="inlineStr">
@@ -22374,12 +22374,12 @@
     <row r="301" ht="16" customHeight="1">
       <c r="A301" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B301" s="16" t="inlineStr">
         <is>
-          <t>CHM-0300</t>
+          <t>PRD-0028</t>
         </is>
       </c>
       <c r="C301" s="15" t="inlineStr">
@@ -22445,12 +22445,12 @@
     <row r="302" ht="16" customHeight="1">
       <c r="A302" s="9" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B302" s="10" t="inlineStr">
         <is>
-          <t>CHM-0301</t>
+          <t>PRD-0029</t>
         </is>
       </c>
       <c r="C302" s="9" t="inlineStr">
@@ -22737,12 +22737,12 @@
     <row r="306" ht="16" customHeight="1">
       <c r="A306" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B306" s="10" t="inlineStr">
         <is>
-          <t>CHM-0305</t>
+          <t>PRD-0030</t>
         </is>
       </c>
       <c r="C306" s="9" t="inlineStr">
@@ -23333,12 +23333,12 @@
     <row r="314" ht="16" customHeight="1">
       <c r="A314" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B314" s="10" t="inlineStr">
         <is>
-          <t>CHM-0313</t>
+          <t>PRD-0031</t>
         </is>
       </c>
       <c r="C314" s="9" t="inlineStr">
@@ -23404,12 +23404,12 @@
     <row r="315" ht="16" customHeight="1">
       <c r="A315" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B315" s="16" t="inlineStr">
         <is>
-          <t>CHM-0314</t>
+          <t>PRD-0032</t>
         </is>
       </c>
       <c r="C315" s="15" t="inlineStr">
@@ -23475,12 +23475,12 @@
     <row r="316" ht="16" customHeight="1">
       <c r="A316" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B316" s="10" t="inlineStr">
         <is>
-          <t>CHM-0315</t>
+          <t>PRD-0033</t>
         </is>
       </c>
       <c r="C316" s="9" t="inlineStr">
@@ -23546,12 +23546,12 @@
     <row r="317" ht="16" customHeight="1">
       <c r="A317" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B317" s="16" t="inlineStr">
         <is>
-          <t>CHM-0316</t>
+          <t>PRD-0034</t>
         </is>
       </c>
       <c r="C317" s="15" t="inlineStr">
@@ -23838,12 +23838,12 @@
     <row r="321" ht="16" customHeight="1">
       <c r="A321" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B321" s="16" t="inlineStr">
         <is>
-          <t>CHM-0320</t>
+          <t>PRD-0035</t>
         </is>
       </c>
       <c r="C321" s="15" t="inlineStr">
@@ -24284,12 +24284,12 @@
     <row r="327" ht="16" customHeight="1">
       <c r="A327" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B327" s="16" t="inlineStr">
         <is>
-          <t>CHM-0326</t>
+          <t>PRD-0036</t>
         </is>
       </c>
       <c r="C327" s="15" t="inlineStr">
@@ -24505,12 +24505,12 @@
     <row r="330" ht="16" customHeight="1">
       <c r="A330" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B330" s="10" t="inlineStr">
         <is>
-          <t>CHM-0329</t>
+          <t>PRD-0037</t>
         </is>
       </c>
       <c r="C330" s="9" t="inlineStr">
@@ -24722,12 +24722,12 @@
     <row r="333" ht="16" customHeight="1">
       <c r="A333" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B333" s="16" t="inlineStr">
         <is>
-          <t>CHM-0332</t>
+          <t>PRD-0038</t>
         </is>
       </c>
       <c r="C333" s="15" t="inlineStr">
@@ -24868,12 +24868,12 @@
     <row r="335" ht="16" customHeight="1">
       <c r="A335" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B335" s="16" t="inlineStr">
         <is>
-          <t>CHM-0334</t>
+          <t>PRD-0039</t>
         </is>
       </c>
       <c r="C335" s="15" t="inlineStr">
@@ -25089,12 +25089,12 @@
     <row r="338" ht="16" customHeight="1">
       <c r="A338" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B338" s="10" t="inlineStr">
         <is>
-          <t>CHM-0337</t>
+          <t>PRD-0040</t>
         </is>
       </c>
       <c r="C338" s="9" t="inlineStr">
@@ -25160,12 +25160,12 @@
     <row r="339" ht="16" customHeight="1">
       <c r="A339" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B339" s="16" t="inlineStr">
         <is>
-          <t>CHM-0338</t>
+          <t>PRD-0041</t>
         </is>
       </c>
       <c r="C339" s="15" t="inlineStr">
@@ -25231,12 +25231,12 @@
     <row r="340" ht="16" customHeight="1">
       <c r="A340" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B340" s="10" t="inlineStr">
         <is>
-          <t>CHM-0339</t>
+          <t>PRD-0042</t>
         </is>
       </c>
       <c r="C340" s="9" t="inlineStr">
@@ -25377,12 +25377,12 @@
     <row r="342" ht="16" customHeight="1">
       <c r="A342" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B342" s="10" t="inlineStr">
         <is>
-          <t>CHM-0341</t>
+          <t>PRD-0043</t>
         </is>
       </c>
       <c r="C342" s="9" t="inlineStr">
@@ -25811,12 +25811,12 @@
     <row r="348" ht="16" customHeight="1">
       <c r="A348" s="9" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B348" s="10" t="inlineStr">
         <is>
-          <t>CHM-0347</t>
+          <t>PRD-0044</t>
         </is>
       </c>
       <c r="C348" s="9" t="inlineStr">
@@ -25882,12 +25882,12 @@
     <row r="349" ht="16" customHeight="1">
       <c r="A349" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B349" s="16" t="inlineStr">
         <is>
-          <t>CHM-0348</t>
+          <t>PRD-0045</t>
         </is>
       </c>
       <c r="C349" s="15" t="inlineStr">
@@ -25953,12 +25953,12 @@
     <row r="350" ht="16" customHeight="1">
       <c r="A350" s="9" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B350" s="10" t="inlineStr">
         <is>
-          <t>CHM-0349</t>
+          <t>PRD-0046</t>
         </is>
       </c>
       <c r="C350" s="9" t="inlineStr">
@@ -26024,12 +26024,12 @@
     <row r="351" ht="16" customHeight="1">
       <c r="A351" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B351" s="16" t="inlineStr">
         <is>
-          <t>CHM-0350</t>
+          <t>PRD-0047</t>
         </is>
       </c>
       <c r="C351" s="15" t="inlineStr">
@@ -26095,12 +26095,12 @@
     <row r="352" ht="16" customHeight="1">
       <c r="A352" s="9" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B352" s="10" t="inlineStr">
         <is>
-          <t>CHM-0351</t>
+          <t>PRD-0048</t>
         </is>
       </c>
       <c r="C352" s="9" t="inlineStr">
@@ -49277,12 +49277,12 @@
     <row r="678" ht="16" customHeight="1">
       <c r="A678" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B678" s="10" t="inlineStr">
         <is>
-          <t>PRD-0001</t>
+          <t>PRD-0049</t>
         </is>
       </c>
       <c r="C678" s="9" t="inlineStr">
@@ -49340,12 +49340,12 @@
     <row r="679" ht="16" customHeight="1">
       <c r="A679" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B679" s="16" t="inlineStr">
         <is>
-          <t>PRD-0002</t>
+          <t>PRD-0050</t>
         </is>
       </c>
       <c r="C679" s="15" t="inlineStr">
@@ -49403,12 +49403,12 @@
     <row r="680" ht="16" customHeight="1">
       <c r="A680" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B680" s="10" t="inlineStr">
         <is>
-          <t>PRD-0003</t>
+          <t>PRD-0051</t>
         </is>
       </c>
       <c r="C680" s="9" t="inlineStr">
@@ -49466,12 +49466,12 @@
     <row r="681" ht="16" customHeight="1">
       <c r="A681" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B681" s="16" t="inlineStr">
         <is>
-          <t>PRD-0004</t>
+          <t>PRD-0052</t>
         </is>
       </c>
       <c r="C681" s="15" t="inlineStr">
@@ -49600,12 +49600,12 @@
     <row r="683" ht="16" customHeight="1">
       <c r="A683" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B683" s="16" t="inlineStr">
         <is>
-          <t>PRD-0006</t>
+          <t>PRD-0053</t>
         </is>
       </c>
       <c r="C683" s="15" t="inlineStr">
@@ -49789,12 +49789,12 @@
     <row r="686" ht="16" customHeight="1">
       <c r="A686" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B686" s="10" t="inlineStr">
         <is>
-          <t>PRD-0009</t>
+          <t>PRD-0054</t>
         </is>
       </c>
       <c r="C686" s="9" t="inlineStr">
@@ -49852,12 +49852,12 @@
     <row r="687" ht="16" customHeight="1">
       <c r="A687" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B687" s="16" t="inlineStr">
         <is>
-          <t>PRD-0010</t>
+          <t>PRD-0055</t>
         </is>
       </c>
       <c r="C687" s="15" t="inlineStr">
@@ -49915,12 +49915,12 @@
     <row r="688" ht="16" customHeight="1">
       <c r="A688" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B688" s="10" t="inlineStr">
         <is>
-          <t>PRD-0011</t>
+          <t>PRD-0056</t>
         </is>
       </c>
       <c r="C688" s="9" t="inlineStr">
@@ -49978,12 +49978,12 @@
     <row r="689" ht="16" customHeight="1">
       <c r="A689" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B689" s="16" t="inlineStr">
         <is>
-          <t>PRD-0012</t>
+          <t>PRD-0057</t>
         </is>
       </c>
       <c r="C689" s="15" t="inlineStr">
@@ -50041,12 +50041,12 @@
     <row r="690" ht="16" customHeight="1">
       <c r="A690" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B690" s="10" t="inlineStr">
         <is>
-          <t>PRD-0013</t>
+          <t>PRD-0058</t>
         </is>
       </c>
       <c r="C690" s="9" t="inlineStr">
@@ -50104,12 +50104,12 @@
     <row r="691" ht="16" customHeight="1">
       <c r="A691" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B691" s="16" t="inlineStr">
         <is>
-          <t>PRD-0014</t>
+          <t>PRD-0059</t>
         </is>
       </c>
       <c r="C691" s="15" t="inlineStr">
@@ -50167,12 +50167,12 @@
     <row r="692" ht="16" customHeight="1">
       <c r="A692" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B692" s="10" t="inlineStr">
         <is>
-          <t>PRD-0015</t>
+          <t>PRD-0060</t>
         </is>
       </c>
       <c r="C692" s="9" t="inlineStr">
@@ -50423,12 +50423,12 @@
     <row r="696" ht="16" customHeight="1">
       <c r="A696" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B696" s="10" t="inlineStr">
         <is>
-          <t>PRD-0019</t>
+          <t>PRD-0061</t>
         </is>
       </c>
       <c r="C696" s="9" t="inlineStr">
@@ -50486,12 +50486,12 @@
     <row r="697" ht="16" customHeight="1">
       <c r="A697" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B697" s="16" t="inlineStr">
         <is>
-          <t>PRD-0020</t>
+          <t>PRD-0062</t>
         </is>
       </c>
       <c r="C697" s="15" t="inlineStr">
@@ -50549,12 +50549,12 @@
     <row r="698" ht="16" customHeight="1">
       <c r="A698" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B698" s="10" t="inlineStr">
         <is>
-          <t>PRD-0021</t>
+          <t>PRD-0063</t>
         </is>
       </c>
       <c r="C698" s="9" t="inlineStr">
@@ -50612,12 +50612,12 @@
     <row r="699" ht="16" customHeight="1">
       <c r="A699" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B699" s="16" t="inlineStr">
         <is>
-          <t>PRD-0022</t>
+          <t>PRD-0064</t>
         </is>
       </c>
       <c r="C699" s="15" t="inlineStr">
@@ -50675,12 +50675,12 @@
     <row r="700" ht="16" customHeight="1">
       <c r="A700" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B700" s="10" t="inlineStr">
         <is>
-          <t>PRD-0023</t>
+          <t>PRD-0065</t>
         </is>
       </c>
       <c r="C700" s="9" t="inlineStr">
@@ -50738,12 +50738,12 @@
     <row r="701" ht="16" customHeight="1">
       <c r="A701" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B701" s="16" t="inlineStr">
         <is>
-          <t>PRD-0024</t>
+          <t>PRD-0066</t>
         </is>
       </c>
       <c r="C701" s="15" t="inlineStr">
@@ -50864,12 +50864,12 @@
     <row r="703" ht="16" customHeight="1">
       <c r="A703" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B703" s="16" t="inlineStr">
         <is>
-          <t>PRD-0026</t>
+          <t>PRD-0067</t>
         </is>
       </c>
       <c r="C703" s="15" t="inlineStr">
@@ -50927,12 +50927,12 @@
     <row r="704" ht="16" customHeight="1">
       <c r="A704" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B704" s="10" t="inlineStr">
         <is>
-          <t>PRD-0027</t>
+          <t>PRD-0068</t>
         </is>
       </c>
       <c r="C704" s="9" t="inlineStr">
@@ -50990,12 +50990,12 @@
     <row r="705" ht="16" customHeight="1">
       <c r="A705" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B705" s="16" t="inlineStr">
         <is>
-          <t>PRD-0028</t>
+          <t>PRD-0069</t>
         </is>
       </c>
       <c r="C705" s="15" t="inlineStr">
@@ -51053,12 +51053,12 @@
     <row r="706" ht="16" customHeight="1">
       <c r="A706" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B706" s="10" t="inlineStr">
         <is>
-          <t>PRD-0029</t>
+          <t>PRD-0070</t>
         </is>
       </c>
       <c r="C706" s="9" t="inlineStr">
@@ -51112,12 +51112,12 @@
     <row r="707" ht="16" customHeight="1">
       <c r="A707" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B707" s="16" t="inlineStr">
         <is>
-          <t>PRD-0030</t>
+          <t>PRD-0071</t>
         </is>
       </c>
       <c r="C707" s="15" t="inlineStr">
@@ -51376,12 +51376,12 @@
     <row r="711" ht="16" customHeight="1">
       <c r="A711" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B711" s="16" t="inlineStr">
         <is>
-          <t>PRD-0034</t>
+          <t>PRD-0072</t>
         </is>
       </c>
       <c r="C711" s="15" t="inlineStr">
@@ -51439,12 +51439,12 @@
     <row r="712" ht="16" customHeight="1">
       <c r="A712" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B712" s="10" t="inlineStr">
         <is>
-          <t>PRD-0035</t>
+          <t>PRD-0073</t>
         </is>
       </c>
       <c r="C712" s="9" t="inlineStr">
@@ -51502,12 +51502,12 @@
     <row r="713" ht="16" customHeight="1">
       <c r="A713" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B713" s="16" t="inlineStr">
         <is>
-          <t>PRD-0036</t>
+          <t>PRD-0074</t>
         </is>
       </c>
       <c r="C713" s="15" t="inlineStr">
@@ -51565,12 +51565,12 @@
     <row r="714" ht="16" customHeight="1">
       <c r="A714" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B714" s="10" t="inlineStr">
         <is>
-          <t>PRD-0037</t>
+          <t>PRD-0075</t>
         </is>
       </c>
       <c r="C714" s="9" t="inlineStr">
@@ -51628,12 +51628,12 @@
     <row r="715" ht="16" customHeight="1">
       <c r="A715" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B715" s="16" t="inlineStr">
         <is>
-          <t>PRD-0038</t>
+          <t>PRD-0076</t>
         </is>
       </c>
       <c r="C715" s="15" t="inlineStr">
@@ -51691,12 +51691,12 @@
     <row r="716" ht="16" customHeight="1">
       <c r="A716" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B716" s="10" t="inlineStr">
         <is>
-          <t>PRD-0039</t>
+          <t>PRD-0077</t>
         </is>
       </c>
       <c r="C716" s="9" t="inlineStr">
@@ -51754,12 +51754,12 @@
     <row r="717" ht="16" customHeight="1">
       <c r="A717" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B717" s="16" t="inlineStr">
         <is>
-          <t>PRD-0040</t>
+          <t>PRD-0078</t>
         </is>
       </c>
       <c r="C717" s="15" t="inlineStr">
@@ -51817,12 +51817,12 @@
     <row r="718" ht="16" customHeight="1">
       <c r="A718" s="9" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B718" s="10" t="inlineStr">
         <is>
-          <t>PRD-0041</t>
+          <t>PRD-0079</t>
         </is>
       </c>
       <c r="C718" s="9" t="inlineStr">
@@ -52483,12 +52483,12 @@
     <row r="728" ht="16" customHeight="1">
       <c r="A728" s="9" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B728" s="10" t="inlineStr">
         <is>
-          <t>PRD-0051</t>
+          <t>PRD-0080</t>
         </is>
       </c>
       <c r="C728" s="9" t="inlineStr">
@@ -52546,12 +52546,12 @@
     <row r="729" ht="16" customHeight="1">
       <c r="A729" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B729" s="16" t="inlineStr">
         <is>
-          <t>PRD-0052</t>
+          <t>PRD-0081</t>
         </is>
       </c>
       <c r="C729" s="15" t="inlineStr">
@@ -52609,12 +52609,12 @@
     <row r="730" ht="16" customHeight="1">
       <c r="A730" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B730" s="10" t="inlineStr">
         <is>
-          <t>PRD-0053</t>
+          <t>PRD-0082</t>
         </is>
       </c>
       <c r="C730" s="9" t="inlineStr">
@@ -52672,12 +52672,12 @@
     <row r="731" ht="16" customHeight="1">
       <c r="A731" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B731" s="16" t="inlineStr">
         <is>
-          <t>PRD-0054</t>
+          <t>PRD-0083</t>
         </is>
       </c>
       <c r="C731" s="15" t="inlineStr">
@@ -52735,12 +52735,12 @@
     <row r="732" ht="16" customHeight="1">
       <c r="A732" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B732" s="10" t="inlineStr">
         <is>
-          <t>PRD-0055</t>
+          <t>PRD-0084</t>
         </is>
       </c>
       <c r="C732" s="9" t="inlineStr">
@@ -52798,12 +52798,12 @@
     <row r="733" ht="16" customHeight="1">
       <c r="A733" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B733" s="16" t="inlineStr">
         <is>
-          <t>PRD-0056</t>
+          <t>PRD-0085</t>
         </is>
       </c>
       <c r="C733" s="15" t="inlineStr">
@@ -52861,12 +52861,12 @@
     <row r="734" ht="16" customHeight="1">
       <c r="A734" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B734" s="10" t="inlineStr">
         <is>
-          <t>PRD-0057</t>
+          <t>PRD-0086</t>
         </is>
       </c>
       <c r="C734" s="9" t="inlineStr">
@@ -52924,12 +52924,12 @@
     <row r="735" ht="16" customHeight="1">
       <c r="A735" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B735" s="16" t="inlineStr">
         <is>
-          <t>PRD-0058</t>
+          <t>PRD-0087</t>
         </is>
       </c>
       <c r="C735" s="15" t="inlineStr">
@@ -52987,12 +52987,12 @@
     <row r="736" ht="16" customHeight="1">
       <c r="A736" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B736" s="10" t="inlineStr">
         <is>
-          <t>PRD-0059</t>
+          <t>PRD-0088</t>
         </is>
       </c>
       <c r="C736" s="9" t="inlineStr">
@@ -53050,12 +53050,12 @@
     <row r="737" ht="16" customHeight="1">
       <c r="A737" s="15" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B737" s="16" t="inlineStr">
         <is>
-          <t>PRD-0060</t>
+          <t>PRD-0089</t>
         </is>
       </c>
       <c r="C737" s="15" t="inlineStr">
@@ -53113,12 +53113,12 @@
     <row r="738" ht="16" customHeight="1">
       <c r="A738" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B738" s="10" t="inlineStr">
         <is>
-          <t>PRD-0061</t>
+          <t>PRD-0090</t>
         </is>
       </c>
       <c r="C738" s="9" t="inlineStr">
@@ -53176,12 +53176,12 @@
     <row r="739" ht="16" customHeight="1">
       <c r="A739" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B739" s="16" t="inlineStr">
         <is>
-          <t>PRD-0062</t>
+          <t>PRD-0091</t>
         </is>
       </c>
       <c r="C739" s="15" t="inlineStr">
@@ -53239,12 +53239,12 @@
     <row r="740" ht="16" customHeight="1">
       <c r="A740" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B740" s="10" t="inlineStr">
         <is>
-          <t>PRD-0063</t>
+          <t>PRD-0092</t>
         </is>
       </c>
       <c r="C740" s="9" t="inlineStr">
@@ -53302,12 +53302,12 @@
     <row r="741" ht="16" customHeight="1">
       <c r="A741" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B741" s="16" t="inlineStr">
         <is>
-          <t>PRD-0064</t>
+          <t>PRD-0093</t>
         </is>
       </c>
       <c r="C741" s="15" t="inlineStr">
@@ -53361,12 +53361,12 @@
     <row r="742" ht="16" customHeight="1">
       <c r="A742" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B742" s="10" t="inlineStr">
         <is>
-          <t>PRD-0065</t>
+          <t>PRD-0094</t>
         </is>
       </c>
       <c r="C742" s="9" t="inlineStr">
@@ -53420,12 +53420,12 @@
     <row r="743" ht="16" customHeight="1">
       <c r="A743" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B743" s="16" t="inlineStr">
         <is>
-          <t>PRD-0066</t>
+          <t>PRD-0095</t>
         </is>
       </c>
       <c r="C743" s="15" t="inlineStr">
@@ -53483,12 +53483,12 @@
     <row r="744" ht="16" customHeight="1">
       <c r="A744" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B744" s="10" t="inlineStr">
         <is>
-          <t>PRD-0067</t>
+          <t>PRD-0096</t>
         </is>
       </c>
       <c r="C744" s="9" t="inlineStr">
@@ -53546,12 +53546,12 @@
     <row r="745" ht="16" customHeight="1">
       <c r="A745" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B745" s="16" t="inlineStr">
         <is>
-          <t>PRD-0068</t>
+          <t>PRD-0097</t>
         </is>
       </c>
       <c r="C745" s="15" t="inlineStr">
@@ -53609,12 +53609,12 @@
     <row r="746" ht="16" customHeight="1">
       <c r="A746" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B746" s="10" t="inlineStr">
         <is>
-          <t>PRD-0069</t>
+          <t>PRD-0098</t>
         </is>
       </c>
       <c r="C746" s="9" t="inlineStr">
@@ -53672,12 +53672,12 @@
     <row r="747" ht="16" customHeight="1">
       <c r="A747" s="15" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B747" s="16" t="inlineStr">
         <is>
-          <t>PRD-0070</t>
+          <t>PRD-0099</t>
         </is>
       </c>
       <c r="C747" s="15" t="inlineStr">
@@ -53991,12 +53991,12 @@
     <row r="752" ht="16" customHeight="1">
       <c r="A752" s="9" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B752" s="10" t="inlineStr">
         <is>
-          <t>PRD-0075</t>
+          <t>PRD-0100</t>
         </is>
       </c>
       <c r="C752" s="9" t="inlineStr">
@@ -54054,12 +54054,12 @@
     <row r="753" ht="16" customHeight="1">
       <c r="A753" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B753" s="16" t="inlineStr">
         <is>
-          <t>PRD-0076</t>
+          <t>PRD-0101</t>
         </is>
       </c>
       <c r="C753" s="15" t="inlineStr">
@@ -54117,12 +54117,12 @@
     <row r="754" ht="16" customHeight="1">
       <c r="A754" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B754" s="10" t="inlineStr">
         <is>
-          <t>PRD-0077</t>
+          <t>PRD-0102</t>
         </is>
       </c>
       <c r="C754" s="9" t="inlineStr">
@@ -54180,12 +54180,12 @@
     <row r="755" ht="16" customHeight="1">
       <c r="A755" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B755" s="16" t="inlineStr">
         <is>
-          <t>PRD-0078</t>
+          <t>PRD-0103</t>
         </is>
       </c>
       <c r="C755" s="15" t="inlineStr">
@@ -54239,12 +54239,12 @@
     <row r="756" ht="16" customHeight="1">
       <c r="A756" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B756" s="10" t="inlineStr">
         <is>
-          <t>PRD-0079</t>
+          <t>PRD-0104</t>
         </is>
       </c>
       <c r="C756" s="9" t="inlineStr">
@@ -54302,12 +54302,12 @@
     <row r="757" ht="16" customHeight="1">
       <c r="A757" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B757" s="16" t="inlineStr">
         <is>
-          <t>PRD-0080</t>
+          <t>PRD-0105</t>
         </is>
       </c>
       <c r="C757" s="15" t="inlineStr">
@@ -54361,12 +54361,12 @@
     <row r="758" ht="16" customHeight="1">
       <c r="A758" s="9" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B758" s="10" t="inlineStr">
         <is>
-          <t>PRD-0081</t>
+          <t>PRD-0106</t>
         </is>
       </c>
       <c r="C758" s="9" t="inlineStr">
@@ -54487,12 +54487,12 @@
     <row r="760" ht="16" customHeight="1">
       <c r="A760" s="9" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B760" s="10" t="inlineStr">
         <is>
-          <t>PRD-0083</t>
+          <t>PRD-0107</t>
         </is>
       </c>
       <c r="C760" s="9" t="inlineStr">
@@ -54550,12 +54550,12 @@
     <row r="761" ht="16" customHeight="1">
       <c r="A761" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B761" s="16" t="inlineStr">
         <is>
-          <t>PRD-0084</t>
+          <t>PRD-0108</t>
         </is>
       </c>
       <c r="C761" s="15" t="inlineStr">
@@ -55208,12 +55208,12 @@
     <row r="771" ht="16" customHeight="1">
       <c r="A771" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B771" s="16" t="inlineStr">
         <is>
-          <t>PRD-0094</t>
+          <t>PRD-0109</t>
         </is>
       </c>
       <c r="C771" s="15" t="inlineStr">
@@ -55271,12 +55271,12 @@
     <row r="772" ht="16" customHeight="1">
       <c r="A772" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B772" s="10" t="inlineStr">
         <is>
-          <t>PRD-0095</t>
+          <t>PRD-0110</t>
         </is>
       </c>
       <c r="C772" s="9" t="inlineStr">
@@ -55334,12 +55334,12 @@
     <row r="773" ht="16" customHeight="1">
       <c r="A773" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B773" s="16" t="inlineStr">
         <is>
-          <t>PRD-0096</t>
+          <t>PRD-0111</t>
         </is>
       </c>
       <c r="C773" s="15" t="inlineStr">
@@ -55397,12 +55397,12 @@
     <row r="774" ht="16" customHeight="1">
       <c r="A774" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B774" s="10" t="inlineStr">
         <is>
-          <t>PRD-0097</t>
+          <t>PRD-0112</t>
         </is>
       </c>
       <c r="C774" s="9" t="inlineStr">
@@ -55460,12 +55460,12 @@
     <row r="775" ht="16" customHeight="1">
       <c r="A775" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B775" s="16" t="inlineStr">
         <is>
-          <t>PRD-0098</t>
+          <t>PRD-0113</t>
         </is>
       </c>
       <c r="C775" s="15" t="inlineStr">
@@ -55523,12 +55523,12 @@
     <row r="776" ht="16" customHeight="1">
       <c r="A776" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B776" s="10" t="inlineStr">
         <is>
-          <t>PRD-0099</t>
+          <t>PRD-0114</t>
         </is>
       </c>
       <c r="C776" s="9" t="inlineStr">
@@ -55586,12 +55586,12 @@
     <row r="777" ht="16" customHeight="1">
       <c r="A777" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B777" s="16" t="inlineStr">
         <is>
-          <t>PRD-0100</t>
+          <t>PRD-0115</t>
         </is>
       </c>
       <c r="C777" s="15" t="inlineStr">
@@ -55649,12 +55649,12 @@
     <row r="778" ht="16" customHeight="1">
       <c r="A778" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B778" s="10" t="inlineStr">
         <is>
-          <t>PRD-0101</t>
+          <t>PRD-0116</t>
         </is>
       </c>
       <c r="C778" s="9" t="inlineStr">
@@ -55712,12 +55712,12 @@
     <row r="779" ht="16" customHeight="1">
       <c r="A779" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B779" s="16" t="inlineStr">
         <is>
-          <t>PRD-0102</t>
+          <t>PRD-0117</t>
         </is>
       </c>
       <c r="C779" s="15" t="inlineStr">
@@ -55775,12 +55775,12 @@
     <row r="780" ht="16" customHeight="1">
       <c r="A780" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B780" s="10" t="inlineStr">
         <is>
-          <t>PRD-0103</t>
+          <t>PRD-0118</t>
         </is>
       </c>
       <c r="C780" s="9" t="inlineStr">
@@ -55838,12 +55838,12 @@
     <row r="781" ht="16" customHeight="1">
       <c r="A781" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B781" s="16" t="inlineStr">
         <is>
-          <t>PRD-0104</t>
+          <t>PRD-0119</t>
         </is>
       </c>
       <c r="C781" s="15" t="inlineStr">
@@ -55901,12 +55901,12 @@
     <row r="782" ht="16" customHeight="1">
       <c r="A782" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B782" s="10" t="inlineStr">
         <is>
-          <t>PRD-0105</t>
+          <t>PRD-0120</t>
         </is>
       </c>
       <c r="C782" s="9" t="inlineStr">
@@ -55964,12 +55964,12 @@
     <row r="783" ht="16" customHeight="1">
       <c r="A783" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B783" s="16" t="inlineStr">
         <is>
-          <t>PRD-0106</t>
+          <t>PRD-0121</t>
         </is>
       </c>
       <c r="C783" s="15" t="inlineStr">
@@ -56027,12 +56027,12 @@
     <row r="784" ht="16" customHeight="1">
       <c r="A784" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B784" s="10" t="inlineStr">
         <is>
-          <t>PRD-0107</t>
+          <t>PRD-0122</t>
         </is>
       </c>
       <c r="C784" s="9" t="inlineStr">
@@ -56291,12 +56291,12 @@
     <row r="788" ht="16" customHeight="1">
       <c r="A788" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B788" s="10" t="inlineStr">
         <is>
-          <t>PRD-0111</t>
+          <t>PRD-0123</t>
         </is>
       </c>
       <c r="C788" s="9" t="inlineStr">
@@ -56354,12 +56354,12 @@
     <row r="789" ht="16" customHeight="1">
       <c r="A789" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B789" s="16" t="inlineStr">
         <is>
-          <t>PRD-0112</t>
+          <t>PRD-0124</t>
         </is>
       </c>
       <c r="C789" s="15" t="inlineStr">
@@ -56417,12 +56417,12 @@
     <row r="790" ht="16" customHeight="1">
       <c r="A790" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B790" s="10" t="inlineStr">
         <is>
-          <t>PRD-0113</t>
+          <t>PRD-0125</t>
         </is>
       </c>
       <c r="C790" s="9" t="inlineStr">
@@ -56480,12 +56480,12 @@
     <row r="791" ht="16" customHeight="1">
       <c r="A791" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B791" s="16" t="inlineStr">
         <is>
-          <t>PRD-0114</t>
+          <t>PRD-0126</t>
         </is>
       </c>
       <c r="C791" s="15" t="inlineStr">
@@ -56543,12 +56543,12 @@
     <row r="792" ht="16" customHeight="1">
       <c r="A792" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B792" s="10" t="inlineStr">
         <is>
-          <t>PRD-0115</t>
+          <t>PRD-0127</t>
         </is>
       </c>
       <c r="C792" s="9" t="inlineStr">
@@ -56602,12 +56602,12 @@
     <row r="793" ht="16" customHeight="1">
       <c r="A793" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B793" s="16" t="inlineStr">
         <is>
-          <t>PRD-0116</t>
+          <t>PRD-0128</t>
         </is>
       </c>
       <c r="C793" s="15" t="inlineStr">
@@ -56661,12 +56661,12 @@
     <row r="794" ht="16" customHeight="1">
       <c r="A794" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B794" s="10" t="inlineStr">
         <is>
-          <t>PRD-0117</t>
+          <t>PRD-0129</t>
         </is>
       </c>
       <c r="C794" s="9" t="inlineStr">
@@ -56720,12 +56720,12 @@
     <row r="795" ht="16" customHeight="1">
       <c r="A795" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B795" s="16" t="inlineStr">
         <is>
-          <t>PRD-0118</t>
+          <t>PRD-0130</t>
         </is>
       </c>
       <c r="C795" s="15" t="inlineStr">
@@ -56779,12 +56779,12 @@
     <row r="796" ht="16" customHeight="1">
       <c r="A796" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B796" s="10" t="inlineStr">
         <is>
-          <t>PRD-0119</t>
+          <t>PRD-0131</t>
         </is>
       </c>
       <c r="C796" s="9" t="inlineStr">
@@ -56842,12 +56842,12 @@
     <row r="797" ht="16" customHeight="1">
       <c r="A797" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B797" s="16" t="inlineStr">
         <is>
-          <t>PRD-0120</t>
+          <t>PRD-0132</t>
         </is>
       </c>
       <c r="C797" s="15" t="inlineStr">
@@ -56905,12 +56905,12 @@
     <row r="798" ht="16" customHeight="1">
       <c r="A798" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B798" s="10" t="inlineStr">
         <is>
-          <t>PRD-0121</t>
+          <t>PRD-0133</t>
         </is>
       </c>
       <c r="C798" s="9" t="inlineStr">
@@ -56968,12 +56968,12 @@
     <row r="799" ht="16" customHeight="1">
       <c r="A799" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B799" s="16" t="inlineStr">
         <is>
-          <t>PRD-0122</t>
+          <t>PRD-0134</t>
         </is>
       </c>
       <c r="C799" s="15" t="inlineStr">
@@ -57457,12 +57457,12 @@
     <row r="806" ht="16" customHeight="1">
       <c r="A806" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B806" s="10" t="inlineStr">
         <is>
-          <t>PRD-0129</t>
+          <t>PRD-0135</t>
         </is>
       </c>
       <c r="C806" s="9" t="inlineStr">
@@ -58820,12 +58820,12 @@
     <row r="827" ht="16" customHeight="1">
       <c r="A827" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B827" s="16" t="inlineStr">
         <is>
-          <t>PRD-0150</t>
+          <t>PRD-0136</t>
         </is>
       </c>
       <c r="C827" s="15" t="inlineStr">
@@ -58883,12 +58883,12 @@
     <row r="828" ht="16" customHeight="1">
       <c r="A828" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B828" s="10" t="inlineStr">
         <is>
-          <t>PRD-0151</t>
+          <t>PRD-0137</t>
         </is>
       </c>
       <c r="C828" s="9" t="inlineStr">
@@ -58946,12 +58946,12 @@
     <row r="829" ht="16" customHeight="1">
       <c r="A829" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B829" s="16" t="inlineStr">
         <is>
-          <t>PRD-0152</t>
+          <t>PRD-0138</t>
         </is>
       </c>
       <c r="C829" s="15" t="inlineStr">
@@ -59009,12 +59009,12 @@
     <row r="830" ht="16" customHeight="1">
       <c r="A830" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B830" s="10" t="inlineStr">
         <is>
-          <t>PRD-0153</t>
+          <t>PRD-0139</t>
         </is>
       </c>
       <c r="C830" s="9" t="inlineStr">
@@ -59072,12 +59072,12 @@
     <row r="831" ht="16" customHeight="1">
       <c r="A831" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B831" s="16" t="inlineStr">
         <is>
-          <t>PRD-0154</t>
+          <t>PRD-0140</t>
         </is>
       </c>
       <c r="C831" s="15" t="inlineStr">
@@ -59135,12 +59135,12 @@
     <row r="832" ht="16" customHeight="1">
       <c r="A832" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B832" s="10" t="inlineStr">
         <is>
-          <t>PRD-0155</t>
+          <t>PRD-0141</t>
         </is>
       </c>
       <c r="C832" s="9" t="inlineStr">
@@ -59198,12 +59198,12 @@
     <row r="833" ht="16" customHeight="1">
       <c r="A833" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B833" s="16" t="inlineStr">
         <is>
-          <t>PRD-0156</t>
+          <t>PRD-0142</t>
         </is>
       </c>
       <c r="C833" s="15" t="inlineStr">
@@ -59261,12 +59261,12 @@
     <row r="834" ht="16" customHeight="1">
       <c r="A834" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B834" s="10" t="inlineStr">
         <is>
-          <t>PRD-0157</t>
+          <t>PRD-0143</t>
         </is>
       </c>
       <c r="C834" s="9" t="inlineStr">
@@ -59324,12 +59324,12 @@
     <row r="835" ht="16" customHeight="1">
       <c r="A835" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B835" s="16" t="inlineStr">
         <is>
-          <t>PRD-0158</t>
+          <t>PRD-0144</t>
         </is>
       </c>
       <c r="C835" s="15" t="inlineStr">
@@ -59387,12 +59387,12 @@
     <row r="836" ht="16" customHeight="1">
       <c r="A836" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B836" s="10" t="inlineStr">
         <is>
-          <t>PRD-0159</t>
+          <t>PRD-0145</t>
         </is>
       </c>
       <c r="C836" s="9" t="inlineStr">
@@ -59450,12 +59450,12 @@
     <row r="837" ht="16" customHeight="1">
       <c r="A837" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B837" s="16" t="inlineStr">
         <is>
-          <t>PRD-0160</t>
+          <t>PRD-0146</t>
         </is>
       </c>
       <c r="C837" s="15" t="inlineStr">
@@ -59513,12 +59513,12 @@
     <row r="838" ht="16" customHeight="1">
       <c r="A838" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B838" s="10" t="inlineStr">
         <is>
-          <t>PRD-0161</t>
+          <t>PRD-0147</t>
         </is>
       </c>
       <c r="C838" s="9" t="inlineStr">
@@ -59576,12 +59576,12 @@
     <row r="839" ht="16" customHeight="1">
       <c r="A839" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B839" s="16" t="inlineStr">
         <is>
-          <t>PRD-0162</t>
+          <t>PRD-0148</t>
         </is>
       </c>
       <c r="C839" s="15" t="inlineStr">
@@ -59639,12 +59639,12 @@
     <row r="840" ht="16" customHeight="1">
       <c r="A840" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B840" s="10" t="inlineStr">
         <is>
-          <t>PRD-0163</t>
+          <t>PRD-0149</t>
         </is>
       </c>
       <c r="C840" s="9" t="inlineStr">
@@ -59966,12 +59966,12 @@
     <row r="845" ht="16" customHeight="1">
       <c r="A845" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B845" s="16" t="inlineStr">
         <is>
-          <t>PRD-0168</t>
+          <t>PRD-0150</t>
         </is>
       </c>
       <c r="C845" s="15" t="inlineStr">
@@ -60025,12 +60025,12 @@
     <row r="846" ht="16" customHeight="1">
       <c r="A846" s="9" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B846" s="10" t="inlineStr">
         <is>
-          <t>PRD-0169</t>
+          <t>PRD-0151</t>
         </is>
       </c>
       <c r="C846" s="9" t="inlineStr">
@@ -60088,12 +60088,12 @@
     <row r="847" ht="16" customHeight="1">
       <c r="A847" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B847" s="16" t="inlineStr">
         <is>
-          <t>PRD-0170</t>
+          <t>PRD-0152</t>
         </is>
       </c>
       <c r="C847" s="15" t="inlineStr">
@@ -60151,12 +60151,12 @@
     <row r="848" ht="16" customHeight="1">
       <c r="A848" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B848" s="10" t="inlineStr">
         <is>
-          <t>PRD-0171</t>
+          <t>PRD-0153</t>
         </is>
       </c>
       <c r="C848" s="9" t="inlineStr">
@@ -60214,12 +60214,12 @@
     <row r="849" ht="16" customHeight="1">
       <c r="A849" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B849" s="16" t="inlineStr">
         <is>
-          <t>PRD-0172</t>
+          <t>PRD-0154</t>
         </is>
       </c>
       <c r="C849" s="15" t="inlineStr">
@@ -60277,12 +60277,12 @@
     <row r="850" ht="16" customHeight="1">
       <c r="A850" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B850" s="10" t="inlineStr">
         <is>
-          <t>PRD-0173</t>
+          <t>PRD-0155</t>
         </is>
       </c>
       <c r="C850" s="9" t="inlineStr">
@@ -60340,12 +60340,12 @@
     <row r="851" ht="16" customHeight="1">
       <c r="A851" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B851" s="16" t="inlineStr">
         <is>
-          <t>PRD-0174</t>
+          <t>PRD-0156</t>
         </is>
       </c>
       <c r="C851" s="15" t="inlineStr">
@@ -60403,12 +60403,12 @@
     <row r="852" ht="16" customHeight="1">
       <c r="A852" s="9" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B852" s="10" t="inlineStr">
         <is>
-          <t>PRD-0175</t>
+          <t>PRD-0157</t>
         </is>
       </c>
       <c r="C852" s="9" t="inlineStr">
@@ -60466,12 +60466,12 @@
     <row r="853" ht="16" customHeight="1">
       <c r="A853" s="15" t="inlineStr">
         <is>
-          <t>Kit/Assay</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B853" s="16" t="inlineStr">
         <is>
-          <t>PRD-0176</t>
+          <t>PRD-0158</t>
         </is>
       </c>
       <c r="C853" s="15" t="inlineStr">
@@ -60529,12 +60529,12 @@
     <row r="854" ht="16" customHeight="1">
       <c r="A854" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B854" s="10" t="inlineStr">
         <is>
-          <t>PRD-0177</t>
+          <t>PRD-0159</t>
         </is>
       </c>
       <c r="C854" s="9" t="inlineStr">
@@ -60592,12 +60592,12 @@
     <row r="855" ht="16" customHeight="1">
       <c r="A855" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B855" s="16" t="inlineStr">
         <is>
-          <t>PRD-0178</t>
+          <t>PRD-0160</t>
         </is>
       </c>
       <c r="C855" s="15" t="inlineStr">
@@ -60718,12 +60718,12 @@
     <row r="857" ht="16" customHeight="1">
       <c r="A857" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B857" s="16" t="inlineStr">
         <is>
-          <t>PRD-0180</t>
+          <t>PRD-0161</t>
         </is>
       </c>
       <c r="C857" s="15" t="inlineStr">
@@ -60781,12 +60781,12 @@
     <row r="858" ht="16" customHeight="1">
       <c r="A858" s="9" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B858" s="10" t="inlineStr">
         <is>
-          <t>PRD-0181</t>
+          <t>PRD-0162</t>
         </is>
       </c>
       <c r="C858" s="9" t="inlineStr">
@@ -60844,12 +60844,12 @@
     <row r="859" ht="16" customHeight="1">
       <c r="A859" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B859" s="16" t="inlineStr">
         <is>
-          <t>PRD-0182</t>
+          <t>PRD-0163</t>
         </is>
       </c>
       <c r="C859" s="15" t="inlineStr">
@@ -60907,12 +60907,12 @@
     <row r="860" ht="16" customHeight="1">
       <c r="A860" s="9" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B860" s="10" t="inlineStr">
         <is>
-          <t>PRD-0183</t>
+          <t>PRD-0164</t>
         </is>
       </c>
       <c r="C860" s="9" t="inlineStr">
@@ -60970,12 +60970,12 @@
     <row r="861" ht="16" customHeight="1">
       <c r="A861" s="15" t="inlineStr">
         <is>
-          <t>Cell Culture</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B861" s="16" t="inlineStr">
         <is>
-          <t>PRD-0184</t>
+          <t>PRD-0165</t>
         </is>
       </c>
       <c r="C861" s="15" t="inlineStr">
@@ -61037,12 +61037,12 @@
     <row r="862" ht="16" customHeight="1">
       <c r="A862" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B862" s="10" t="inlineStr">
         <is>
-          <t>PRD-0185</t>
+          <t>PRD-0166</t>
         </is>
       </c>
       <c r="C862" s="9" t="inlineStr">
@@ -61100,12 +61100,12 @@
     <row r="863" ht="16" customHeight="1">
       <c r="A863" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B863" s="16" t="inlineStr">
         <is>
-          <t>PRD-0186</t>
+          <t>PRD-0167</t>
         </is>
       </c>
       <c r="C863" s="15" t="inlineStr">
@@ -61163,12 +61163,12 @@
     <row r="864" ht="16" customHeight="1">
       <c r="A864" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B864" s="10" t="inlineStr">
         <is>
-          <t>PRD-0187</t>
+          <t>PRD-0168</t>
         </is>
       </c>
       <c r="C864" s="9" t="inlineStr">
@@ -61226,12 +61226,12 @@
     <row r="865" ht="16" customHeight="1">
       <c r="A865" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B865" s="16" t="inlineStr">
         <is>
-          <t>PRD-0188</t>
+          <t>PRD-0169</t>
         </is>
       </c>
       <c r="C865" s="15" t="inlineStr">
@@ -61289,12 +61289,12 @@
     <row r="866" ht="16" customHeight="1">
       <c r="A866" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B866" s="10" t="inlineStr">
         <is>
-          <t>PRD-0189</t>
+          <t>PRD-0170</t>
         </is>
       </c>
       <c r="C866" s="9" t="inlineStr">
@@ -61352,12 +61352,12 @@
     <row r="867" ht="16" customHeight="1">
       <c r="A867" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B867" s="16" t="inlineStr">
         <is>
-          <t>PRD-0190</t>
+          <t>PRD-0171</t>
         </is>
       </c>
       <c r="C867" s="15" t="inlineStr">
@@ -61415,12 +61415,12 @@
     <row r="868" ht="16" customHeight="1">
       <c r="A868" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B868" s="10" t="inlineStr">
         <is>
-          <t>PRD-0191</t>
+          <t>PRD-0172</t>
         </is>
       </c>
       <c r="C868" s="9" t="inlineStr">
@@ -61478,12 +61478,12 @@
     <row r="869" ht="16" customHeight="1">
       <c r="A869" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B869" s="16" t="inlineStr">
         <is>
-          <t>PRD-0192</t>
+          <t>PRD-0173</t>
         </is>
       </c>
       <c r="C869" s="15" t="inlineStr">
@@ -61817,12 +61817,12 @@
     <row r="874" ht="16" customHeight="1">
       <c r="A874" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B874" s="10" t="inlineStr">
         <is>
-          <t>PRD-0197</t>
+          <t>PRD-0174</t>
         </is>
       </c>
       <c r="C874" s="9" t="inlineStr">
@@ -61880,12 +61880,12 @@
     <row r="875" ht="16" customHeight="1">
       <c r="A875" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B875" s="16" t="inlineStr">
         <is>
-          <t>PRD-0198</t>
+          <t>PRD-0175</t>
         </is>
       </c>
       <c r="C875" s="15" t="inlineStr">
@@ -61943,12 +61943,12 @@
     <row r="876" ht="16" customHeight="1">
       <c r="A876" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B876" s="10" t="inlineStr">
         <is>
-          <t>PRD-0199</t>
+          <t>PRD-0176</t>
         </is>
       </c>
       <c r="C876" s="9" t="inlineStr">
@@ -62006,12 +62006,12 @@
     <row r="877" ht="16" customHeight="1">
       <c r="A877" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B877" s="16" t="inlineStr">
         <is>
-          <t>PRD-0200</t>
+          <t>PRD-0177</t>
         </is>
       </c>
       <c r="C877" s="15" t="inlineStr">
@@ -62069,12 +62069,12 @@
     <row r="878" ht="16" customHeight="1">
       <c r="A878" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B878" s="10" t="inlineStr">
         <is>
-          <t>PRD-0201</t>
+          <t>PRD-0178</t>
         </is>
       </c>
       <c r="C878" s="9" t="inlineStr">
@@ -62132,12 +62132,12 @@
     <row r="879" ht="16" customHeight="1">
       <c r="A879" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B879" s="16" t="inlineStr">
         <is>
-          <t>PRD-0202</t>
+          <t>PRD-0179</t>
         </is>
       </c>
       <c r="C879" s="15" t="inlineStr">
@@ -62191,12 +62191,12 @@
     <row r="880" ht="16" customHeight="1">
       <c r="A880" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B880" s="10" t="inlineStr">
         <is>
-          <t>PRD-0203</t>
+          <t>PRD-0180</t>
         </is>
       </c>
       <c r="C880" s="9" t="inlineStr">
@@ -62254,12 +62254,12 @@
     <row r="881" ht="16" customHeight="1">
       <c r="A881" s="15" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B881" s="16" t="inlineStr">
         <is>
-          <t>PRD-0204</t>
+          <t>PRD-0181</t>
         </is>
       </c>
       <c r="C881" s="15" t="inlineStr">
@@ -62317,12 +62317,12 @@
     <row r="882" ht="16" customHeight="1">
       <c r="A882" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="B882" s="10" t="inlineStr">
         <is>
-          <t>PRD-0205</t>
+          <t>PRD-0182</t>
         </is>
       </c>
       <c r="C882" s="9" t="inlineStr">

</xml_diff>